<commit_message>
added scrpit to take wrong data from NSE website and fixed mistake in fo.py
</commit_message>
<xml_diff>
--- a/fo high low.xlsx
+++ b/fo high low.xlsx
@@ -27,24 +27,27 @@
     <t>CLOSE</t>
   </si>
   <si>
+    <t>VOL</t>
+  </si>
+  <si>
+    <t>9:25 CLOSE</t>
+  </si>
+  <si>
+    <t>BN</t>
+  </si>
+  <si>
+    <t>NIFTY</t>
+  </si>
+  <si>
     <t>LTP</t>
   </si>
   <si>
-    <t>VOL</t>
-  </si>
-  <si>
-    <t>9:25 CLOSE</t>
-  </si>
-  <si>
     <t>ADANI</t>
   </si>
   <si>
     <t>AURO</t>
   </si>
   <si>
-    <t>BN</t>
-  </si>
-  <si>
     <t>CANBK</t>
   </si>
   <si>
@@ -58,9 +61,6 @@
   </si>
   <si>
     <t>JIND</t>
-  </si>
-  <si>
-    <t>NIFTY</t>
   </si>
   <si>
     <t>REL</t>
@@ -471,36 +471,60 @@
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
+        <v>5</v>
+      </c>
+      <c r="B2" s="1">
+        <v>52486.45</v>
+      </c>
+      <c r="C2" s="2">
+        <v>52035.45</v>
+      </c>
+      <c r="D2" s="1">
+        <v>52345</v>
+      </c>
+      <c r="E2" s="1">
+        <v>52364.45</v>
+      </c>
+      <c r="F2" s="1">
+        <v>15</v>
+      </c>
+      <c r="G2" s="1">
+        <v>52372.35</v>
+      </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
+        <v>6</v>
+      </c>
+      <c r="B3" s="1">
+        <v>24367.95</v>
+      </c>
+      <c r="C3" s="2">
+        <v>24112</v>
+      </c>
+      <c r="D3" s="1">
+        <v>24318.25</v>
+      </c>
+      <c r="E3" s="1">
+        <v>24304.15</v>
+      </c>
+      <c r="F3" s="1">
+        <v>65</v>
+      </c>
+      <c r="G3" s="1">
+        <v>24130</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -524,18 +548,18 @@
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="2"/>
@@ -546,7 +570,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="2"/>
@@ -557,7 +581,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="2"/>
@@ -568,7 +592,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="2"/>
@@ -579,7 +603,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="2"/>
@@ -590,7 +614,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="2"/>
@@ -601,7 +625,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="2"/>
@@ -612,7 +636,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="2"/>
@@ -623,7 +647,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="B10" s="1"/>
       <c r="C10" s="2"/>

</xml_diff>